<commit_message>
seattle timeline map and other changes
</commit_message>
<xml_diff>
--- a/figures/timeline-sea/TimelineJS3 Template_Seattle DWO_May 2026.xlsx
+++ b/figures/timeline-sea/TimelineJS3 Template_Seattle DWO_May 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lians\git\dwbr-website\figures\timeline-sea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67599B92-4D58-410C-B57B-637714910C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64306BEA-21FB-436A-A8AD-3FB5B0DD219D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="53">
   <si>
     <t>Year</t>
   </si>
@@ -403,13 +403,16 @@
     <t>img/photo_3.jpg</t>
   </si>
   <si>
-    <t>img/photo_4.jpg</t>
-  </si>
-  <si>
     <t>img/photo_7.jpg</t>
   </si>
   <si>
     <t>img/photo_8.jpg</t>
+  </si>
+  <si>
+    <t>img/photo_5.jpg</t>
+  </si>
+  <si>
+    <t>img/photo_4.png</t>
   </si>
 </sst>
 </file>
@@ -1124,9 +1127,6 @@
       <c r="K2" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="20" t="s">
-        <v>47</v>
-      </c>
       <c r="M2" s="21"/>
       <c r="N2" s="21"/>
       <c r="O2" s="12"/>
@@ -1173,7 +1173,9 @@
       <c r="K3" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="L3" s="25"/>
+      <c r="L3" s="20" t="s">
+        <v>47</v>
+      </c>
       <c r="M3" s="25" t="s">
         <v>28</v>
       </c>
@@ -1258,7 +1260,7 @@
         <v>34</v>
       </c>
       <c r="L5" s="34" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="M5" s="28" t="s">
         <v>35</v>
@@ -1300,7 +1302,9 @@
       <c r="K6" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="L6" s="28"/>
+      <c r="L6" s="28" t="s">
+        <v>51</v>
+      </c>
       <c r="M6" s="28" t="s">
         <v>38</v>
       </c>
@@ -1383,7 +1387,7 @@
         <v>43</v>
       </c>
       <c r="L8" s="34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M8" s="28" t="s">
         <v>44</v>
@@ -1426,7 +1430,7 @@
         <v>46</v>
       </c>
       <c r="L9" s="34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="M9" s="28" t="s">
         <v>44</v>
@@ -1466,7 +1470,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="L2" r:id="rId1" display="https://www.flickr.com/photos/139186991@N03/53098748328/in/dateposted-public/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="L3" r:id="rId1" display="https://www.flickr.com/photos/139186991@N03/53098748328/in/dateposted-public/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="S3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="L4" r:id="rId3" display="https://www.flickr.com/photos/197507288@N06/53136362437/in/dateposted-public/" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="L5" r:id="rId4" display="https://www.flickr.com/photos/139186991@N03/53098462054/in/dateposted-public/" xr:uid="{00000000-0004-0000-0000-000003000000}"/>

</xml_diff>